<commit_message>
RPA + Conversational AI customer service prototype
</commit_message>
<xml_diff>
--- a/data/MockCRM_ApplianceOrders.xlsx
+++ b/data/MockCRM_ApplianceOrders.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Orders" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="AuditLog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="EscalationQueue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EscalationQueue" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -676,7 +676,6 @@
           <t>402 Sunshine CHS, Kothrud, Pune 411038</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -846,7 +845,6 @@
           <t>55 Satellite Road, Ahmedabad 380015</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1003,12 +1001,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Delivered</t>
+          <t>Refund Initiated</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1074,7 +1072,6 @@
           <t>14 MG Road, Kochi 682016</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1186,7 +1183,6 @@
           <t>6 Vijayanagar, Mysuru 570017</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1298,7 +1294,6 @@
           <t>11 Linking Road, Bandra, Mumbai 400050</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1526,7 +1521,6 @@
           <t>29 Alkapuri, Vadodara 390007</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1683,12 +1677,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Delivered</t>
+          <t>Refund Initiated</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1713,7 +1707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1774,6 +1768,136 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-16 08:15:40</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4521</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>order.status</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9628</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>READ_STATUS</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Status read: Delivered</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>UiPath Robot</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-16 08:15:41</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4521</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>order.refund</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8866000000000001</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PROCESS_REFUND</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Refund of Rs 2,499.00 initiated.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>RF6484</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>UiPath Robot</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-16 08:15:41</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4509</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>order.refund</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PROCESS_REFUND</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Refund of Rs 4,299.00 initiated.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>RF9432</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>UiPath Robot</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1785,7 +1909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1852,6 +1976,147 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-16 08:15:40</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>order.complaint</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1908</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>LOW_CONFIDENCE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>The message could not be classified confidently (best guess: order.complaint at 0.19). Entities detected: none. Read the customer's message, confirm what they need, and if this phrasing is a common one, add it to the training data so the classifier handles it next time.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Something's wrong with my stuff</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-16 08:15:41</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4516</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>order.refund</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>order_id=4516; amount=72990.0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SENSITIVITY_CAP</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>The order IS marked refund-eligible and all automated checks pass. Recommended action: approve the Rs 72,990.00 refund. This case is above the cap for authorisation reasons only, not because anything looks wrong. Order 4516 - Haier 596L Side by Side (Refrigerator), Rs 72,990.00, status 'Delivered', refund-eligible: Y. Customer: Lakshmi Subramanian (9840556677).</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>I want a refund for order 4516</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-16 08:15:41</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>order.complaint</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.7403</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>category=Washing Machine</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>POLICY_INTENT</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Product complaint - policy routes every complaint to a person. Acknowledge the issue, determine whether this is a replacement, a repair visit or a refund, and set expectations on timing.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>my washing machine arrived broken and it wont start</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>